<commit_message>
add paper and installation instructions, fix bug with finance theme score
</commit_message>
<xml_diff>
--- a/tests/Test case.xlsx
+++ b/tests/Test case.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\danielpert\circulytics_calculator\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1EDD23-03B3-48AF-B7A6-6189A378EE9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{430CD8FE-1651-471A-BFE0-FFD09F312D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{7CEE43CF-3C6E-49A2-BCEF-B05159AE5C5C}"/>
+    <workbookView xWindow="-103" yWindow="18411" windowWidth="33120" windowHeight="9635" activeTab="1" xr2:uid="{7CEE43CF-3C6E-49A2-BCEF-B05159AE5C5C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Example 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Example 2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="79">
   <si>
     <t>Theme 1</t>
   </si>
@@ -231,6 +232,48 @@
   </si>
   <si>
     <t>Overall Score</t>
+  </si>
+  <si>
+    <t>Finance Category</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Lending</t>
+  </si>
+  <si>
+    <t>Fixed Income</t>
+  </si>
+  <si>
+    <t>Private equity</t>
+  </si>
+  <si>
+    <t>Listed equity</t>
+  </si>
+  <si>
+    <t>Real estate</t>
+  </si>
+  <si>
+    <t>11b percentage</t>
+  </si>
+  <si>
+    <t>11a percentage</t>
+  </si>
+  <si>
+    <t>11a weighted percentage</t>
+  </si>
+  <si>
+    <t>11b weighted percentage</t>
+  </si>
+  <si>
+    <t>11a score</t>
+  </si>
+  <si>
+    <t>11b score</t>
+  </si>
+  <si>
+    <t>Theme 11 score</t>
   </si>
 </sst>
 </file>
@@ -1693,4 +1736,197 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36372848-6ABA-4116-9DAA-B9AC844E3E02}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="14.26171875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.05078125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.05078125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2">
+        <v>1000</v>
+      </c>
+      <c r="C2">
+        <f>B2/SUM($B$2:$B$6)</f>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <f>C2*D2</f>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <f>C2*F2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C6" si="0">B3/SUM($B$2:$B$6)</f>
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E6" si="1">C3*D3</f>
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G6" si="2">C3*F3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4">
+        <v>2000</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="D4">
+        <v>0.5</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="2"/>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5">
+        <v>2000</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="F5">
+        <v>0.5</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="2"/>
+        <v>0.14285714285714285</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6">
+        <v>2000</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>0.2857142857142857</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="D7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7">
+        <f>SUM(E2:E6)</f>
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7">
+        <f>SUM(G2:G6)</f>
+        <v>0.71428571428571419</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8">
+        <f>AVERAGE(E7,G7)</f>
+        <v>0.64285714285714279</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>